<commit_message>
Remove incorrect Top 10 Creditors sheet
No purchase/accounts-payable data in uploaded files — only sales and
collections (debtor-side). Added a note to the Summary Dashboard.

https://claude.ai/code/session_01CtMYMSCg9adm625M7g1rVn
</commit_message>
<xml_diff>
--- a/Debtors_Creditors_Sales_Collection_Report.xlsx
+++ b/Debtors_Creditors_Sales_Collection_Report.xlsx
@@ -9,12 +9,11 @@
   <sheets>
     <sheet name="Summary Dashboard" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Top 10 Debtors" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Top 10 Creditors" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Party-wise Summary" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="April Sales Detail" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="May Sales Detail" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="April Collections" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="May Collections" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Party-wise Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="April Sales Detail" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="May Sales Detail" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="April Collections" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="May Collections" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -75,8 +74,13 @@
       <color rgb="00FFFFFF"/>
       <sz val="12"/>
     </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -143,6 +147,11 @@
         <fgColor rgb="00EDE0F5"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEEEE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -184,7 +193,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -303,6 +312,9 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -669,7 +681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -683,7 +695,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>POLYSIL IRRIGATION — SALES &amp; COLLECTION SUMMARY  |  APR–MAY 2026</t>
+          <t>POLYSIL IRRIGATION — DEBTORS, SALES &amp; COLLECTION SUMMARY  |  APR–MAY 2026</t>
         </is>
       </c>
     </row>
@@ -826,8 +838,16 @@
       <c r="E11" s="7" t="n"/>
       <c r="F11" s="7" t="n"/>
     </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="45" t="inlineStr">
+        <is>
+          <t>NOTE: Creditors report could not be prepared — no purchase / accounts-payable data in the provided files.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
+    <mergeCell ref="A13:F13"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
@@ -1231,396 +1251,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="22" t="inlineStr">
-        <is>
-          <t>TOP 10 CREDITORS — Highest Collection Parties (Apr–May 2026)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Ranked by total collections; negative outstanding = advance/excess received vs sales billed</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="23" t="inlineStr">
-        <is>
-          <t>Rank</t>
-        </is>
-      </c>
-      <c r="B3" s="23" t="inlineStr">
-        <is>
-          <t>Party Name</t>
-        </is>
-      </c>
-      <c r="C3" s="23" t="inlineStr">
-        <is>
-          <t>Apr Sales</t>
-        </is>
-      </c>
-      <c r="D3" s="23" t="inlineStr">
-        <is>
-          <t>May Sales</t>
-        </is>
-      </c>
-      <c r="E3" s="23" t="inlineStr">
-        <is>
-          <t>Total Sales</t>
-        </is>
-      </c>
-      <c r="F3" s="23" t="inlineStr">
-        <is>
-          <t>Apr Collection</t>
-        </is>
-      </c>
-      <c r="G3" s="23" t="inlineStr">
-        <is>
-          <t>May Collection</t>
-        </is>
-      </c>
-      <c r="H3" s="23" t="inlineStr">
-        <is>
-          <t>Outstanding</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>Anita Soni</t>
-        </is>
-      </c>
-      <c r="C4" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D4" s="14" t="n">
-        <v>2253926.5</v>
-      </c>
-      <c r="E4" s="14" t="n">
-        <v>2253926.5</v>
-      </c>
-      <c r="F4" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" s="14" t="n">
-        <v>3000000</v>
-      </c>
-      <c r="H4" s="24" t="n">
-        <v>-746073.5</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="25" t="n">
-        <v>2</v>
-      </c>
-      <c r="B5" s="26" t="inlineStr">
-        <is>
-          <t>Pragati Irrigation</t>
-        </is>
-      </c>
-      <c r="C5" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="D5" s="27" t="n">
-        <v>1003334</v>
-      </c>
-      <c r="E5" s="27" t="n">
-        <v>1003334</v>
-      </c>
-      <c r="F5" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" s="27" t="n">
-        <v>1504900</v>
-      </c>
-      <c r="H5" s="24" t="n">
-        <v>-501566</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>ANDRA PRADESH MICRO IRRIGATION PROJECT</t>
-        </is>
-      </c>
-      <c r="C6" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="14" t="n">
-        <v>1343075.52</v>
-      </c>
-      <c r="G6" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" s="24" t="n">
-        <v>-1343075.52</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="25" t="n">
-        <v>4</v>
-      </c>
-      <c r="B7" s="26" t="inlineStr">
-        <is>
-          <t>ROKDE AGRO AGENCY-JAFRABAD</t>
-        </is>
-      </c>
-      <c r="C7" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" s="27" t="n">
-        <v>593919.4</v>
-      </c>
-      <c r="E7" s="27" t="n">
-        <v>593919.4</v>
-      </c>
-      <c r="F7" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" s="27" t="n">
-        <v>800000</v>
-      </c>
-      <c r="H7" s="24" t="n">
-        <v>-206080.6</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Maharudra Agro Agency-Deulgaon Raja</t>
-        </is>
-      </c>
-      <c r="C8" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" s="14" t="n">
-        <v>782700</v>
-      </c>
-      <c r="E8" s="14" t="n">
-        <v>782700</v>
-      </c>
-      <c r="F8" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="14" t="n">
-        <v>795300</v>
-      </c>
-      <c r="H8" s="24" t="n">
-        <v>-12600</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="25" t="n">
-        <v>6</v>
-      </c>
-      <c r="B9" s="26" t="inlineStr">
-        <is>
-          <t>SAI TRADERS</t>
-        </is>
-      </c>
-      <c r="C9" s="27" t="n">
-        <v>161904</v>
-      </c>
-      <c r="D9" s="27" t="n">
-        <v>869050</v>
-      </c>
-      <c r="E9" s="27" t="n">
-        <v>1030954</v>
-      </c>
-      <c r="F9" s="27" t="n">
-        <v>403800</v>
-      </c>
-      <c r="G9" s="27" t="n">
-        <v>384300</v>
-      </c>
-      <c r="H9" s="15" t="n">
-        <v>242854</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>SHRI DATTA KRUPA AGRO AGENCY-KOLGAON</t>
-        </is>
-      </c>
-      <c r="C10" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="14" t="n">
-        <v>1173379.2</v>
-      </c>
-      <c r="E10" s="14" t="n">
-        <v>1173379.2</v>
-      </c>
-      <c r="F10" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="14" t="n">
-        <v>757800</v>
-      </c>
-      <c r="H10" s="15" t="n">
-        <v>415579.2</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="25" t="n">
-        <v>8</v>
-      </c>
-      <c r="B11" s="26" t="inlineStr">
-        <is>
-          <t>Rajesh Singh Thakur</t>
-        </is>
-      </c>
-      <c r="C11" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="27" t="n">
-        <v>740000</v>
-      </c>
-      <c r="G11" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" s="24" t="n">
-        <v>-740000</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>JANAI ENTERPRISES-JAMNER</t>
-        </is>
-      </c>
-      <c r="C12" s="14" t="n">
-        <v>329815</v>
-      </c>
-      <c r="D12" s="14" t="n">
-        <v>477251.7</v>
-      </c>
-      <c r="E12" s="14" t="n">
-        <v>807066.7</v>
-      </c>
-      <c r="F12" s="14" t="n">
-        <v>300000</v>
-      </c>
-      <c r="G12" s="14" t="n">
-        <v>400000</v>
-      </c>
-      <c r="H12" s="15" t="n">
-        <v>107066.7</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="25" t="n">
-        <v>10</v>
-      </c>
-      <c r="B13" s="26" t="inlineStr">
-        <is>
-          <t>Brajesh Kumar Upadhyay</t>
-        </is>
-      </c>
-      <c r="C13" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="27" t="n">
-        <v>696941</v>
-      </c>
-      <c r="G13" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" s="24" t="n">
-        <v>-696941</v>
-      </c>
-    </row>
-    <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="28" t="n"/>
-      <c r="B14" s="29" t="inlineStr">
-        <is>
-          <t>GRAND TOTAL</t>
-        </is>
-      </c>
-      <c r="C14" s="30" t="n">
-        <v>491719</v>
-      </c>
-      <c r="D14" s="30" t="n">
-        <v>7153560.800000001</v>
-      </c>
-      <c r="E14" s="30" t="n">
-        <v>7645279.800000001</v>
-      </c>
-      <c r="F14" s="30" t="n">
-        <v>3483816.52</v>
-      </c>
-      <c r="G14" s="30" t="n">
-        <v>7642300</v>
-      </c>
-      <c r="H14" s="30" t="n">
-        <v>-3480836.72</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:H1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:I146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -6159,7 +5789,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6905,7 +6535,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7859,7 +7489,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8215,7 +7845,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>